<commit_message>
fix(pdf/c9): PDF 가로 방향 강제 — 작업 3
PDF 가 세로로 나오던 문제 해결. 이중 경로 모두 수정.

1) save-all → convertXlsxToPdf (주된 경로, Google Drive API)
   · generateMethodWorkbook 에서 양 시트 (갑지/을지) 에
     pageSetup.orientation='landscape' 명시 강제
   · paperSize=9 (A4), fitToPage=true, fitToWidth=1
   · exceljs readFile 이 템플릿 pageSetup 유실해도 writeBuffer 전
     enforceLandscape() 헬퍼로 재설정
   · Google Sheets 변환 시 xlsx pageSetup 존중 → PDF 가로 보장

2) generate → generatePdfBuffer (puppeteer, e2e 경로)
   · page.pdf({ landscape: true, ... }) 추가

검증:
- samples/ 3개 xlsx 재생성 후 verify-landscape.ts 확인
- Sheet1/Sheet2 모두 orientation=landscape paperSize=9 fitToPage=true 적용 확인
- tests 477/477, build 성공
</commit_message>
<xml_diff>
--- a/samples/sample-1-basic-8rows.xlsx
+++ b/samples/sample-1-basic-8rows.xlsx
@@ -3228,14 +3228,18 @@
     <mergeCell ref="B19:C22"/>
     <mergeCell ref="D19:R22"/>
   </mergeCells>
+  <printOptions horizontalCentered="1"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0" footer="0"/>
-  <pageSetup paperSize="9" orientation="landscape" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1" firstPageNumber="1" useFirstPageNumber="1" copies="1"/>
+  <pageSetup paperSize="9" orientation="landscape" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="0" firstPageNumber="1" useFirstPageNumber="1" copies="1"/>
   <drawing r:id="rId1"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <sheetPr>
+    <pageSetUpPr fitToPage="1"/>
+  </sheetPr>
   <dimension ref="A1:R21"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="0" defaultColWidth="12.63"/>
   <cols>
@@ -3805,8 +3809,9 @@
     <mergeCell ref="J5:K5"/>
     <mergeCell ref="L5:M5"/>
   </mergeCells>
+  <printOptions horizontalCentered="1"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0" footer="0"/>
-  <pageSetup paperSize="9" orientation="landscape" horizontalDpi="4294967295" verticalDpi="4294967295" scale="71" fitToWidth="1" fitToHeight="1" firstPageNumber="1" useFirstPageNumber="1" copies="1"/>
+  <pageSetup paperSize="9" orientation="landscape" horizontalDpi="4294967295" verticalDpi="4294967295" scale="71" fitToWidth="1" fitToHeight="0" firstPageNumber="1" useFirstPageNumber="1" copies="1"/>
   <drawing r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
test(excel/c8): UAT 샘플 3종 재생성 — c10/c11/c12 효과 반영
c10 (fitToHeight=1) + c11 (빈 row15-17 splice + 병합/이미지 보정) +
c12 (행 높이 동적 산정) + c1 commit 의 샘플 total 채움 효과를 모두 반영.

검증:
  - K14/K15/E11 = 합계 정상 표시
  - rowCount: 27 → 24 (3 행 단축)
  - fitToHeight=1: 갑지 단일 페이지
  - 이미지 row 23.05 → 20.06 정확 이동
  - 병합 B19:C22/D19:R22 → B16:C19/D16:R19 정상 갱신
</commit_message>
<xml_diff>
--- a/samples/sample-1-basic-8rows.xlsx
+++ b/samples/sample-1-basic-8rows.xlsx
@@ -93,7 +93,7 @@
 (부가세 별도)</t>
   </si>
   <si>
-    <t>일금 영원 정(₩0)</t>
+    <t>일금 이천사백사십만원 정(₩24,400,000)</t>
   </si>
   <si>
     <t>품 명</t>
@@ -612,7 +612,6 @@
       <sz val="12"/>
       <name val="Arial"/>
     </font>
-    <font/>
     <font>
       <b/>
       <color theme="1"/>
@@ -643,6 +642,7 @@
       <sz val="11"/>
       <name val="Arial"/>
     </font>
+    <font/>
     <font>
       <color theme="1"/>
       <sz val="12"/>
@@ -687,7 +687,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="58">
+  <borders count="42">
     <border>
       <left/>
       <right/>
@@ -820,19 +820,6 @@
         <color rgb="FFCCCCCC"/>
       </left>
       <right/>
-      <top style="thick">
-        <color rgb="FF000000"/>
-      </top>
-      <bottom style="thin">
-        <color rgb="FFB7B7B7"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right style="thin">
-        <color rgb="FF747474"/>
-      </right>
       <top style="thick">
         <color rgb="FF000000"/>
       </top>
@@ -881,28 +868,6 @@
       <diagonal/>
     </border>
     <border>
-      <left/>
-      <right style="thin">
-        <color rgb="FF747474"/>
-      </right>
-      <top style="thick">
-        <color rgb="FF000000"/>
-      </top>
-      <bottom/>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right style="thin">
-        <color rgb="FF525979"/>
-      </right>
-      <top style="thick">
-        <color rgb="FF000000"/>
-      </top>
-      <bottom/>
-      <diagonal/>
-    </border>
-    <border>
       <left style="thin">
         <color rgb="FFCCCCCC"/>
       </left>
@@ -916,30 +881,6 @@
         <color rgb="FFB7B7B7"/>
       </left>
       <right/>
-      <top style="thin">
-        <color rgb="FFB7B7B7"/>
-      </top>
-      <bottom style="thin">
-        <color rgb="FFB7B7B7"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right/>
-      <top style="thin">
-        <color rgb="FFB7B7B7"/>
-      </top>
-      <bottom style="thin">
-        <color rgb="FFB7B7B7"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right style="thin">
-        <color rgb="FFB7B7B7"/>
-      </right>
       <top style="thin">
         <color rgb="FFB7B7B7"/>
       </top>
@@ -975,65 +916,6 @@
       <diagonal/>
     </border>
     <border>
-      <left/>
-      <right style="thin">
-        <color rgb="FFCCCCCC"/>
-      </right>
-      <top/>
-      <bottom style="thin">
-        <color rgb="FFCCCCCC"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color rgb="FFCCCCCC"/>
-      </left>
-      <right/>
-      <top style="thin">
-        <color rgb="FFB7B7B7"/>
-      </top>
-      <bottom style="thin">
-        <color rgb="FFCCCCCC"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right/>
-      <top style="thin">
-        <color rgb="FFB7B7B7"/>
-      </top>
-      <bottom style="thin">
-        <color rgb="FFCCCCCC"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right style="thin">
-        <color rgb="FFB7B7B7"/>
-      </right>
-      <top style="thin">
-        <color rgb="FFB7B7B7"/>
-      </top>
-      <bottom style="thin">
-        <color rgb="FFCCCCCC"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color rgb="FFCCCCCC"/>
-      </left>
-      <right/>
-      <top style="thin">
-        <color rgb="FFCCCCCC"/>
-      </top>
-      <bottom/>
-      <diagonal/>
-    </border>
-    <border>
       <left style="thin">
         <color rgb="FFCCCCCC"/>
       </left>
@@ -1047,32 +929,6 @@
       <diagonal/>
     </border>
     <border>
-      <left/>
-      <right style="thin">
-        <color rgb="FFCCCCCC"/>
-      </right>
-      <top style="thin">
-        <color rgb="FFCCCCCC"/>
-      </top>
-      <bottom style="thin">
-        <color rgb="FFCCCCCC"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right style="thin">
-        <color rgb="FFB7B7B7"/>
-      </right>
-      <top style="thin">
-        <color rgb="FFCCCCCC"/>
-      </top>
-      <bottom style="thin">
-        <color rgb="FFCCCCCC"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
       <left style="thin">
         <color rgb="FFB7B7B7"/>
       </left>
@@ -1086,16 +942,14 @@
       <diagonal/>
     </border>
     <border>
-      <left/>
-      <right style="thin">
+      <left style="thin">
         <color rgb="FFCCCCCC"/>
-      </right>
+      </left>
+      <right/>
       <top style="thin">
         <color rgb="FFCCCCCC"/>
       </top>
-      <bottom style="thin">
-        <color rgb="FFB7B7B7"/>
-      </bottom>
+      <bottom/>
       <diagonal/>
     </border>
     <border>
@@ -1107,66 +961,6 @@
         <color rgb="FFB7B7B7"/>
       </top>
       <bottom/>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right/>
-      <top style="thin">
-        <color rgb="FFB7B7B7"/>
-      </top>
-      <bottom/>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right style="thin">
-        <color rgb="FFB7B7B7"/>
-      </right>
-      <top style="thin">
-        <color rgb="FFB7B7B7"/>
-      </top>
-      <bottom/>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color rgb="FFB7B7B7"/>
-      </left>
-      <right/>
-      <top/>
-      <bottom/>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right style="thin">
-        <color rgb="FFB7B7B7"/>
-      </right>
-      <top/>
-      <bottom/>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color rgb="FFB7B7B7"/>
-      </left>
-      <right/>
-      <top/>
-      <bottom style="thin">
-        <color rgb="FFB7B7B7"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right style="thin">
-        <color rgb="FFB7B7B7"/>
-      </right>
-      <top/>
-      <bottom style="thin">
-        <color rgb="FFB7B7B7"/>
-      </bottom>
       <diagonal/>
     </border>
     <border>
@@ -1210,6 +1004,17 @@
       <left style="thin">
         <color rgb="FF747474"/>
       </left>
+      <right style="thin">
+        <color rgb="FF747474"/>
+      </right>
+      <top style="thick">
+        <color rgb="FF000000"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
       <right style="thin">
         <color rgb="FF747474"/>
       </right>
@@ -1342,6 +1147,17 @@
       <diagonal/>
     </border>
     <border>
+      <left/>
+      <right style="thin">
+        <color rgb="FFB7B7B7"/>
+      </right>
+      <top/>
+      <bottom style="thin">
+        <color rgb="FFB7B7B7"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
       <left style="thin">
         <color rgb="FFCCCCCC"/>
       </left>
@@ -1358,7 +1174,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="132">
+  <cellXfs count="99">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
@@ -1391,282 +1207,239 @@
     <xf numFmtId="0" fontId="5" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" shrinkToFit="1"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="7" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="6" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="6" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="7" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="2" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="7" fillId="2" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="164" fontId="5" fillId="0" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" shrinkToFit="1"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="7" fillId="4" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="6" fillId="4" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="2" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="6" fillId="2" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" shrinkToFit="1"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="3" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="7" fillId="3" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" shrinkToFit="1"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="7" fillId="4" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="6" fillId="4" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="2" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="6" fillId="2" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" shrinkToFit="1"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="7" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="8" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="7" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="165" fontId="9" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="165" fontId="8" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1" shrinkToFit="1"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="8" fillId="3" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="7" fillId="3" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="8" fillId="3" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="7" fillId="3" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="3" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="7" fillId="3" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="3" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="7" fillId="3" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="18" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="8" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="7" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="19" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="21" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="18" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="22" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="23" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="24" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="19" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="3" fontId="5" fillId="0" borderId="18" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="3" fontId="5" fillId="0" borderId="21" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="25" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="26" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="27" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="28" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="29" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="30" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="30" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="21" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="31" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="32" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="33" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="5" fillId="5" borderId="31" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="5" borderId="34" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="35" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="5" fillId="5" borderId="31" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="3" fontId="5" fillId="5" borderId="21" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="30" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="36" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="37" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="38" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="39" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="40" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="25" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="41" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="42" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="right"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="43" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="43" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="44" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="8" fillId="3" borderId="45" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="3" borderId="46" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="3" borderId="47" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="48" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="8" fillId="3" borderId="49" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="3" borderId="50" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="3" borderId="51" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="3" borderId="52" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="3" borderId="53" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="3" borderId="54" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="55" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="56" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="42" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="3" fontId="5" fillId="0" borderId="42" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="166" fontId="5" fillId="0" borderId="42" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="3" fontId="5" fillId="2" borderId="42" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="55" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="42" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="57" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="56" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="6" borderId="21" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="6" borderId="56" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="6" borderId="42" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="3" fontId="5" fillId="6" borderId="42" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="3" fontId="5" fillId="5" borderId="42" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="166" fontId="5" fillId="5" borderId="42" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="5" borderId="42" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="21" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="5" fillId="5" borderId="21" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="5" borderId="56" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="5" borderId="22" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="5" borderId="21" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="3" fontId="5" fillId="5" borderId="18" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="23" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="24" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="25" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="25" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="26" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="7" fillId="3" borderId="27" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="3" borderId="28" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="29" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="7" fillId="3" borderId="30" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="31" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="7" fillId="3" borderId="32" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="3" borderId="33" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="3" borderId="34" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="3" borderId="35" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="3" borderId="36" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="3" borderId="37" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="38" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="39" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="40" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="3" fontId="5" fillId="0" borderId="40" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="166" fontId="5" fillId="0" borderId="40" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="3" fontId="5" fillId="2" borderId="40" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="38" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="40" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="41" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="39" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="6" borderId="18" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="6" borderId="39" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="6" borderId="40" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="3" fontId="5" fillId="6" borderId="40" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="3" fontId="5" fillId="5" borderId="40" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="166" fontId="5" fillId="5" borderId="40" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="5" borderId="40" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="3" fontId="5" fillId="5" borderId="42" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="18" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="5" borderId="18" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="5" borderId="39" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="5" borderId="21" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="3" fontId="5" fillId="5" borderId="40" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="5" borderId="18" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="5" borderId="24" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="5" borderId="19" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="3" fontId="7" fillId="5" borderId="42" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="3" fontId="6" fillId="5" borderId="40" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="5" borderId="42" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="5" borderId="40" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -1692,8 +1465,8 @@
     <xdr:from>
       <xdr:col>6</xdr:col>
       <xdr:colOff>219075</xdr:colOff>
-      <xdr:row>23</xdr:row>
-      <xdr:rowOff>9525</xdr:rowOff>
+      <xdr:row>20</xdr:row>
+      <xdr:rowOff>9524</xdr:rowOff>
     </xdr:from>
     <xdr:ext cx="6562725" cy="466725"/>
     <xdr:pic>
@@ -2012,7 +1785,7 @@
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:AK27"/>
+  <dimension ref="A1:AK24"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="0" defaultColWidth="12.63"/>
   <cols>
     <col min="1" max="1" width="8" customWidth="1"/>
@@ -2041,22 +1814,22 @@
       <c r="B1" s="2" t="s">
         <v>0</v>
       </c>
-      <c r="C1"/>
-      <c r="D1"/>
-      <c r="E1"/>
-      <c r="F1"/>
-      <c r="G1"/>
-      <c r="H1"/>
-      <c r="I1"/>
-      <c r="J1"/>
-      <c r="K1"/>
-      <c r="L1"/>
-      <c r="M1"/>
-      <c r="N1"/>
-      <c r="O1"/>
-      <c r="P1"/>
-      <c r="Q1"/>
-      <c r="R1"/>
+      <c r="C1" s="2"/>
+      <c r="D1" s="2"/>
+      <c r="E1" s="2"/>
+      <c r="F1" s="2"/>
+      <c r="G1" s="2"/>
+      <c r="H1" s="2"/>
+      <c r="I1" s="2"/>
+      <c r="J1" s="2"/>
+      <c r="K1" s="2"/>
+      <c r="L1" s="2"/>
+      <c r="M1" s="2"/>
+      <c r="N1" s="2"/>
+      <c r="O1" s="2"/>
+      <c r="P1" s="2"/>
+      <c r="Q1" s="2"/>
+      <c r="R1" s="2"/>
       <c r="S1" s="1"/>
       <c r="T1" s="1"/>
       <c r="U1" s="1"/>
@@ -2079,23 +1852,23 @@
     </row>
     <row r="2" ht="15" customHeight="1" spans="1:37" x14ac:dyDescent="0.25">
       <c r="A2" s="1"/>
-      <c r="B2"/>
-      <c r="C2"/>
-      <c r="D2"/>
-      <c r="E2"/>
-      <c r="F2"/>
-      <c r="G2"/>
-      <c r="H2"/>
-      <c r="I2"/>
-      <c r="J2"/>
-      <c r="K2"/>
-      <c r="L2"/>
-      <c r="M2"/>
-      <c r="N2"/>
-      <c r="O2"/>
-      <c r="P2"/>
-      <c r="Q2"/>
-      <c r="R2"/>
+      <c r="B2" s="2"/>
+      <c r="C2" s="2"/>
+      <c r="D2" s="2"/>
+      <c r="E2" s="2"/>
+      <c r="F2" s="2"/>
+      <c r="G2" s="2"/>
+      <c r="H2" s="2"/>
+      <c r="I2" s="2"/>
+      <c r="J2" s="2"/>
+      <c r="K2" s="2"/>
+      <c r="L2" s="2"/>
+      <c r="M2" s="2"/>
+      <c r="N2" s="2"/>
+      <c r="O2" s="2"/>
+      <c r="P2" s="2"/>
+      <c r="Q2" s="2"/>
+      <c r="R2" s="2"/>
       <c r="S2" s="1"/>
       <c r="T2" s="1"/>
       <c r="U2" s="1"/>
@@ -2243,32 +2016,32 @@
       <c r="D6" s="13" t="s">
         <v>3</v>
       </c>
-      <c r="E6" s="14"/>
-      <c r="F6" s="14"/>
-      <c r="G6" s="15"/>
-      <c r="H6" s="16" t="s">
+      <c r="E6" s="13"/>
+      <c r="F6" s="13"/>
+      <c r="G6" s="14"/>
+      <c r="H6" s="15" t="s">
         <v>4</v>
       </c>
-      <c r="I6" s="17"/>
-      <c r="J6" s="18" t="s">
+      <c r="I6" s="16"/>
+      <c r="J6" s="17" t="s">
         <v>5</v>
       </c>
-      <c r="K6" s="19"/>
-      <c r="L6" s="16" t="s">
+      <c r="K6" s="17"/>
+      <c r="L6" s="15" t="s">
         <v>6</v>
       </c>
-      <c r="M6" s="17"/>
-      <c r="N6" s="20" t="s">
+      <c r="M6" s="16"/>
+      <c r="N6" s="18" t="s">
         <v>7</v>
       </c>
-      <c r="O6" s="16" t="s">
+      <c r="O6" s="15" t="s">
         <v>8</v>
       </c>
-      <c r="P6" s="17"/>
-      <c r="Q6" s="18" t="s">
+      <c r="P6" s="16"/>
+      <c r="Q6" s="17" t="s">
         <v>9</v>
       </c>
-      <c r="R6" s="19"/>
+      <c r="R6" s="17"/>
       <c r="S6" s="1"/>
       <c r="T6" s="1"/>
       <c r="U6" s="1"/>
@@ -2291,35 +2064,35 @@
     </row>
     <row r="7" ht="26.25" customHeight="1" spans="1:37" x14ac:dyDescent="0.25">
       <c r="A7" s="5"/>
-      <c r="B7" s="21" t="s">
+      <c r="B7" s="19" t="s">
         <v>10</v>
       </c>
-      <c r="C7" s="22"/>
-      <c r="D7" s="23" t="s">
+      <c r="C7" s="20"/>
+      <c r="D7" s="21" t="s">
         <v>11</v>
       </c>
-      <c r="E7" s="24"/>
-      <c r="F7" s="24"/>
-      <c r="G7" s="15"/>
-      <c r="H7" s="25" t="s">
+      <c r="E7" s="21"/>
+      <c r="F7" s="21"/>
+      <c r="G7" s="14"/>
+      <c r="H7" s="22" t="s">
         <v>12</v>
       </c>
-      <c r="I7" s="26"/>
-      <c r="J7" s="27" t="s">
+      <c r="I7" s="23"/>
+      <c r="J7" s="24" t="s">
         <v>13</v>
       </c>
-      <c r="K7" s="28"/>
-      <c r="L7" s="25" t="s">
+      <c r="K7" s="24"/>
+      <c r="L7" s="22" t="s">
         <v>14</v>
       </c>
-      <c r="M7" s="26"/>
-      <c r="N7" s="29" t="s">
+      <c r="M7" s="23"/>
+      <c r="N7" s="25" t="s">
         <v>15</v>
       </c>
-      <c r="O7" s="28"/>
-      <c r="P7" s="28"/>
-      <c r="Q7" s="28"/>
-      <c r="R7" s="28"/>
+      <c r="O7" s="25"/>
+      <c r="P7" s="25"/>
+      <c r="Q7" s="25"/>
+      <c r="R7" s="25"/>
       <c r="S7" s="1"/>
       <c r="T7" s="1"/>
       <c r="U7" s="1"/>
@@ -2342,35 +2115,35 @@
     </row>
     <row r="8" ht="26.25" customHeight="1" spans="1:37" x14ac:dyDescent="0.25">
       <c r="A8" s="5"/>
-      <c r="B8" s="21" t="s">
+      <c r="B8" s="19" t="s">
         <v>16</v>
       </c>
-      <c r="C8" s="22"/>
-      <c r="D8" s="30" t="s">
+      <c r="C8" s="20"/>
+      <c r="D8" s="26" t="s">
         <v>17</v>
       </c>
-      <c r="E8" s="24"/>
-      <c r="F8" s="24"/>
-      <c r="G8" s="15"/>
-      <c r="H8" s="25" t="s">
+      <c r="E8" s="26"/>
+      <c r="F8" s="26"/>
+      <c r="G8" s="14"/>
+      <c r="H8" s="22" t="s">
         <v>18</v>
       </c>
-      <c r="I8" s="26"/>
-      <c r="J8" s="27" t="s">
+      <c r="I8" s="23"/>
+      <c r="J8" s="24" t="s">
         <v>19</v>
       </c>
-      <c r="K8" s="28"/>
-      <c r="L8" s="25" t="s">
+      <c r="K8" s="24"/>
+      <c r="L8" s="22" t="s">
         <v>20</v>
       </c>
-      <c r="M8" s="26"/>
-      <c r="N8" s="29" t="s">
+      <c r="M8" s="23"/>
+      <c r="N8" s="25" t="s">
         <v>21</v>
       </c>
-      <c r="O8" s="28"/>
-      <c r="P8" s="28"/>
-      <c r="Q8" s="28"/>
-      <c r="R8" s="28"/>
+      <c r="O8" s="25"/>
+      <c r="P8" s="25"/>
+      <c r="Q8" s="25"/>
+      <c r="R8" s="25"/>
       <c r="S8" s="1"/>
       <c r="T8" s="1"/>
       <c r="U8" s="1"/>
@@ -2393,31 +2166,31 @@
     </row>
     <row r="9" ht="27.75" customHeight="1" spans="1:37" x14ac:dyDescent="0.25">
       <c r="A9" s="5"/>
-      <c r="B9" s="31" t="s">
+      <c r="B9" s="27" t="s">
         <v>22</v>
       </c>
-      <c r="C9" s="22"/>
-      <c r="D9" s="32" t="s">
+      <c r="C9" s="20"/>
+      <c r="D9" s="28" t="s">
         <v>23</v>
       </c>
-      <c r="E9" s="33"/>
-      <c r="F9" s="33"/>
-      <c r="G9" s="15"/>
-      <c r="H9" s="34" t="s">
+      <c r="E9" s="28"/>
+      <c r="F9" s="28"/>
+      <c r="G9" s="14"/>
+      <c r="H9" s="29" t="s">
         <v>24</v>
       </c>
-      <c r="I9" s="35"/>
-      <c r="J9" s="36" t="s">
+      <c r="I9" s="30"/>
+      <c r="J9" s="31" t="s">
         <v>23</v>
       </c>
-      <c r="K9" s="28"/>
-      <c r="L9" s="28"/>
-      <c r="M9" s="28"/>
-      <c r="N9" s="28"/>
-      <c r="O9" s="28"/>
-      <c r="P9" s="28"/>
-      <c r="Q9" s="28"/>
-      <c r="R9" s="28"/>
+      <c r="K9" s="31"/>
+      <c r="L9" s="31"/>
+      <c r="M9" s="31"/>
+      <c r="N9" s="31"/>
+      <c r="O9" s="31"/>
+      <c r="P9" s="31"/>
+      <c r="Q9" s="31"/>
+      <c r="R9" s="31"/>
       <c r="S9" s="1"/>
       <c r="T9" s="1"/>
       <c r="U9" s="1"/>
@@ -2440,23 +2213,23 @@
     </row>
     <row r="10" ht="17.25" customHeight="1" spans="1:37" x14ac:dyDescent="0.25">
       <c r="A10" s="5"/>
-      <c r="B10" s="37"/>
-      <c r="C10" s="37"/>
-      <c r="D10" s="37"/>
-      <c r="E10" s="38"/>
-      <c r="F10" s="39"/>
-      <c r="G10" s="39"/>
-      <c r="H10" s="39"/>
-      <c r="I10" s="39"/>
-      <c r="J10" s="39"/>
-      <c r="K10" s="39"/>
-      <c r="L10" s="39"/>
-      <c r="M10" s="39"/>
-      <c r="N10" s="39"/>
-      <c r="O10" s="39"/>
-      <c r="P10" s="39"/>
-      <c r="Q10" s="39"/>
-      <c r="R10" s="39"/>
+      <c r="B10" s="32"/>
+      <c r="C10" s="32"/>
+      <c r="D10" s="32"/>
+      <c r="E10" s="33"/>
+      <c r="F10" s="33"/>
+      <c r="G10" s="33"/>
+      <c r="H10" s="33"/>
+      <c r="I10" s="33"/>
+      <c r="J10" s="33"/>
+      <c r="K10" s="33"/>
+      <c r="L10" s="33"/>
+      <c r="M10" s="33"/>
+      <c r="N10" s="33"/>
+      <c r="O10" s="33"/>
+      <c r="P10" s="33"/>
+      <c r="Q10" s="33"/>
+      <c r="R10" s="33"/>
       <c r="S10" s="1"/>
       <c r="T10" s="1"/>
       <c r="U10" s="1"/>
@@ -2479,27 +2252,27 @@
     </row>
     <row r="11" ht="50.25" customHeight="1" spans="1:37" x14ac:dyDescent="0.25">
       <c r="A11" s="5"/>
-      <c r="B11" s="40" t="s">
+      <c r="B11" s="34" t="s">
         <v>25</v>
       </c>
-      <c r="C11" s="41"/>
-      <c r="D11" s="41"/>
-      <c r="E11" s="42" t="s">
+      <c r="C11" s="34"/>
+      <c r="D11" s="34"/>
+      <c r="E11" s="35" t="s">
         <v>26</v>
       </c>
-      <c r="F11" s="41"/>
-      <c r="G11" s="41"/>
-      <c r="H11" s="41"/>
-      <c r="I11" s="41"/>
-      <c r="J11" s="41"/>
-      <c r="K11" s="41"/>
-      <c r="L11" s="41"/>
-      <c r="M11" s="41"/>
-      <c r="N11" s="41"/>
-      <c r="O11" s="41"/>
-      <c r="P11" s="41"/>
-      <c r="Q11" s="41"/>
-      <c r="R11" s="41"/>
+      <c r="F11" s="35"/>
+      <c r="G11" s="35"/>
+      <c r="H11" s="35"/>
+      <c r="I11" s="35"/>
+      <c r="J11" s="35"/>
+      <c r="K11" s="35"/>
+      <c r="L11" s="35"/>
+      <c r="M11" s="35"/>
+      <c r="N11" s="35"/>
+      <c r="O11" s="35"/>
+      <c r="P11" s="35"/>
+      <c r="Q11" s="35"/>
+      <c r="R11" s="35"/>
       <c r="S11" s="1"/>
       <c r="T11" s="1"/>
       <c r="U11" s="1"/>
@@ -2522,23 +2295,23 @@
     </row>
     <row r="12" ht="17.25" customHeight="1" spans="1:37" x14ac:dyDescent="0.25">
       <c r="A12" s="1"/>
-      <c r="B12" s="43"/>
-      <c r="C12" s="43"/>
-      <c r="D12" s="43"/>
-      <c r="E12" s="44"/>
-      <c r="F12" s="45"/>
-      <c r="G12" s="45"/>
-      <c r="H12" s="45"/>
-      <c r="I12" s="45"/>
-      <c r="J12" s="45"/>
-      <c r="K12" s="45"/>
-      <c r="L12" s="45"/>
-      <c r="M12" s="45"/>
-      <c r="N12" s="45"/>
-      <c r="O12" s="45"/>
-      <c r="P12" s="45"/>
-      <c r="Q12" s="45"/>
-      <c r="R12" s="45"/>
+      <c r="B12" s="36"/>
+      <c r="C12" s="36"/>
+      <c r="D12" s="36"/>
+      <c r="E12" s="37"/>
+      <c r="F12" s="37"/>
+      <c r="G12" s="37"/>
+      <c r="H12" s="37"/>
+      <c r="I12" s="37"/>
+      <c r="J12" s="37"/>
+      <c r="K12" s="37"/>
+      <c r="L12" s="37"/>
+      <c r="M12" s="37"/>
+      <c r="N12" s="37"/>
+      <c r="O12" s="37"/>
+      <c r="P12" s="37"/>
+      <c r="Q12" s="37"/>
+      <c r="R12" s="37"/>
       <c r="S12" s="1"/>
       <c r="T12" s="1"/>
       <c r="U12" s="1"/>
@@ -2561,36 +2334,36 @@
     </row>
     <row r="13" ht="29.25" customHeight="1" spans="1:37" x14ac:dyDescent="0.25">
       <c r="A13" s="1"/>
-      <c r="B13" s="46" t="s">
+      <c r="B13" s="38" t="s">
         <v>27</v>
       </c>
-      <c r="C13" s="14"/>
-      <c r="D13" s="14"/>
-      <c r="E13" s="47"/>
-      <c r="F13" s="48" t="s">
+      <c r="C13" s="38"/>
+      <c r="D13" s="38"/>
+      <c r="E13" s="38"/>
+      <c r="F13" s="39" t="s">
         <v>28</v>
       </c>
-      <c r="G13" s="47"/>
-      <c r="H13" s="49" t="s">
+      <c r="G13" s="39"/>
+      <c r="H13" s="40" t="s">
         <v>29</v>
       </c>
-      <c r="I13" s="50" t="s">
+      <c r="I13" s="41" t="s">
         <v>30</v>
       </c>
-      <c r="J13" s="51"/>
-      <c r="K13" s="52" t="s">
+      <c r="J13" s="41"/>
+      <c r="K13" s="42" t="s">
         <v>31</v>
       </c>
-      <c r="L13" s="41"/>
-      <c r="M13" s="41"/>
-      <c r="N13" s="53"/>
-      <c r="O13" s="52" t="s">
+      <c r="L13" s="42"/>
+      <c r="M13" s="42"/>
+      <c r="N13" s="42"/>
+      <c r="O13" s="42" t="s">
         <v>32</v>
       </c>
-      <c r="P13" s="41"/>
-      <c r="Q13" s="41"/>
-      <c r="R13" s="41"/>
-      <c r="S13" s="54"/>
+      <c r="P13" s="42"/>
+      <c r="Q13" s="42"/>
+      <c r="R13" s="42"/>
+      <c r="S13" s="43"/>
       <c r="T13" s="1"/>
       <c r="U13" s="1"/>
       <c r="V13" s="1"/>
@@ -2612,33 +2385,33 @@
     </row>
     <row r="14" ht="28.5" customHeight="1" spans="1:37" x14ac:dyDescent="0.25">
       <c r="A14" s="1"/>
-      <c r="B14" s="55" t="str">
+      <c r="B14" s="44" t="str">
         <f>Sheet2!C3</f>
         <v>옥상 이중복합방수 3.8mm (제 1안)</v>
       </c>
-      <c r="C14" s="56"/>
-      <c r="D14" s="56"/>
-      <c r="E14" s="57"/>
-      <c r="F14" s="55" t="s">
+      <c r="C14" s="44"/>
+      <c r="D14" s="44"/>
+      <c r="E14" s="44"/>
+      <c r="F14" s="44" t="s">
         <v>33</v>
       </c>
-      <c r="G14" s="57"/>
-      <c r="H14" s="58">
+      <c r="G14" s="44"/>
+      <c r="H14" s="45">
         <v>1</v>
       </c>
-      <c r="I14" s="59"/>
-      <c r="J14"/>
-      <c r="K14" s="60">
-        <v>0</v>
-      </c>
-      <c r="L14" s="56"/>
-      <c r="M14" s="56"/>
-      <c r="N14" s="57"/>
-      <c r="O14" s="61"/>
-      <c r="P14" s="33"/>
-      <c r="Q14" s="33"/>
-      <c r="R14" s="62"/>
-      <c r="S14" s="54"/>
+      <c r="I14" s="46"/>
+      <c r="J14" s="46"/>
+      <c r="K14" s="47">
+        <v>24448700</v>
+      </c>
+      <c r="L14" s="47"/>
+      <c r="M14" s="47"/>
+      <c r="N14" s="47"/>
+      <c r="O14" s="48"/>
+      <c r="P14" s="48"/>
+      <c r="Q14" s="48"/>
+      <c r="R14" s="48"/>
+      <c r="S14" s="43"/>
       <c r="T14" s="1"/>
       <c r="U14" s="1"/>
       <c r="V14" s="1"/>
@@ -2658,26 +2431,32 @@
       <c r="AJ14" s="1"/>
       <c r="AK14" s="1"/>
     </row>
-    <row r="15" ht="25.5" customHeight="1" spans="1:37" x14ac:dyDescent="0.25">
+    <row r="15" ht="27" customHeight="1" spans="1:37" x14ac:dyDescent="0.25">
       <c r="A15" s="1"/>
-      <c r="B15" s="63"/>
-      <c r="C15" s="64"/>
-      <c r="D15" s="64"/>
-      <c r="E15" s="65"/>
-      <c r="F15" s="66"/>
-      <c r="G15" s="67"/>
-      <c r="H15" s="68"/>
-      <c r="I15" s="69"/>
-      <c r="J15" s="67"/>
-      <c r="K15" s="70"/>
-      <c r="L15" s="56"/>
-      <c r="M15" s="56"/>
-      <c r="N15" s="57"/>
-      <c r="O15" s="71"/>
-      <c r="P15" s="28"/>
-      <c r="Q15" s="28"/>
-      <c r="R15" s="72"/>
-      <c r="S15" s="54"/>
+      <c r="B15" s="49" t="s">
+        <v>34</v>
+      </c>
+      <c r="C15" s="49"/>
+      <c r="D15" s="49"/>
+      <c r="E15" s="49"/>
+      <c r="F15" s="50"/>
+      <c r="G15" s="50"/>
+      <c r="H15" s="51"/>
+      <c r="I15" s="49"/>
+      <c r="J15" s="49"/>
+      <c r="K15" s="52">
+        <v>24400000</v>
+      </c>
+      <c r="L15" s="52"/>
+      <c r="M15" s="52"/>
+      <c r="N15" s="52"/>
+      <c r="O15" s="49" t="s">
+        <v>35</v>
+      </c>
+      <c r="P15" s="49"/>
+      <c r="Q15" s="49"/>
+      <c r="R15" s="49"/>
+      <c r="S15" s="43"/>
       <c r="T15" s="1"/>
       <c r="U15" s="1"/>
       <c r="V15" s="1"/>
@@ -2697,25 +2476,29 @@
       <c r="AJ15" s="1"/>
       <c r="AK15" s="1"/>
     </row>
-    <row r="16" ht="25.5" customHeight="1" spans="1:37" x14ac:dyDescent="0.25">
+    <row r="16" ht="26.25" customHeight="1" spans="1:37" x14ac:dyDescent="0.25">
       <c r="A16" s="1"/>
-      <c r="B16" s="71"/>
-      <c r="C16" s="28"/>
-      <c r="D16" s="28"/>
-      <c r="E16" s="72"/>
-      <c r="F16" s="71"/>
-      <c r="G16" s="72"/>
-      <c r="H16" s="68"/>
-      <c r="I16" s="71"/>
-      <c r="J16" s="72"/>
-      <c r="K16" s="70"/>
-      <c r="L16" s="56"/>
-      <c r="M16" s="56"/>
-      <c r="N16" s="57"/>
-      <c r="O16" s="71"/>
-      <c r="P16" s="28"/>
-      <c r="Q16" s="28"/>
-      <c r="R16" s="72"/>
+      <c r="B16" s="53" t="s">
+        <v>36</v>
+      </c>
+      <c r="C16" s="53"/>
+      <c r="D16" s="54" t="s">
+        <v>37</v>
+      </c>
+      <c r="E16" s="54"/>
+      <c r="F16" s="54"/>
+      <c r="G16" s="54"/>
+      <c r="H16" s="54"/>
+      <c r="I16" s="54"/>
+      <c r="J16" s="54"/>
+      <c r="K16" s="54"/>
+      <c r="L16" s="54"/>
+      <c r="M16" s="54"/>
+      <c r="N16" s="54"/>
+      <c r="O16" s="54"/>
+      <c r="P16" s="54"/>
+      <c r="Q16" s="54"/>
+      <c r="R16" s="54"/>
       <c r="S16" s="1"/>
       <c r="T16" s="1"/>
       <c r="U16" s="1"/>
@@ -2736,26 +2519,26 @@
       <c r="AJ16" s="1"/>
       <c r="AK16" s="1"/>
     </row>
-    <row r="17" ht="25.5" customHeight="1" spans="1:37" x14ac:dyDescent="0.25">
+    <row r="17" ht="19.5" customHeight="1" spans="1:37" x14ac:dyDescent="0.25">
       <c r="A17" s="1"/>
-      <c r="B17" s="71"/>
-      <c r="C17" s="28"/>
-      <c r="D17" s="28"/>
-      <c r="E17" s="73"/>
-      <c r="F17" s="66"/>
-      <c r="G17" s="67"/>
-      <c r="H17" s="68"/>
-      <c r="I17" s="69"/>
-      <c r="J17" s="67"/>
-      <c r="K17" s="70"/>
-      <c r="L17" s="56"/>
-      <c r="M17" s="56"/>
-      <c r="N17" s="57"/>
-      <c r="O17" s="71"/>
-      <c r="P17" s="28"/>
-      <c r="Q17" s="28"/>
-      <c r="R17" s="72"/>
-      <c r="S17" s="54"/>
+      <c r="B17" s="53"/>
+      <c r="C17" s="53"/>
+      <c r="D17" s="54"/>
+      <c r="E17" s="54"/>
+      <c r="F17" s="54"/>
+      <c r="G17" s="54"/>
+      <c r="H17" s="54"/>
+      <c r="I17" s="54"/>
+      <c r="J17" s="54"/>
+      <c r="K17" s="54"/>
+      <c r="L17" s="54"/>
+      <c r="M17" s="54"/>
+      <c r="N17" s="54"/>
+      <c r="O17" s="54"/>
+      <c r="P17" s="54"/>
+      <c r="Q17" s="54"/>
+      <c r="R17" s="54"/>
+      <c r="S17" s="1"/>
       <c r="T17" s="1"/>
       <c r="U17" s="1"/>
       <c r="V17" s="1"/>
@@ -2775,32 +2558,26 @@
       <c r="AJ17" s="1"/>
       <c r="AK17" s="1"/>
     </row>
-    <row r="18" ht="27" customHeight="1" spans="1:37" x14ac:dyDescent="0.25">
+    <row r="18" ht="21" customHeight="1" spans="1:37" x14ac:dyDescent="0.25">
       <c r="A18" s="1"/>
-      <c r="B18" s="74" t="s">
-        <v>34</v>
-      </c>
-      <c r="C18" s="28"/>
-      <c r="D18" s="28"/>
-      <c r="E18" s="73"/>
-      <c r="F18" s="75"/>
-      <c r="G18" s="76"/>
-      <c r="H18" s="77"/>
-      <c r="I18" s="74"/>
-      <c r="J18" s="28"/>
-      <c r="K18" s="78">
-        <v>0</v>
-      </c>
-      <c r="L18" s="56"/>
-      <c r="M18" s="56"/>
-      <c r="N18" s="57"/>
-      <c r="O18" s="74" t="s">
-        <v>35</v>
-      </c>
-      <c r="P18" s="28"/>
-      <c r="Q18" s="28"/>
-      <c r="R18" s="28"/>
-      <c r="S18" s="54"/>
+      <c r="B18" s="53"/>
+      <c r="C18" s="53"/>
+      <c r="D18" s="54"/>
+      <c r="E18" s="54"/>
+      <c r="F18" s="54"/>
+      <c r="G18" s="54"/>
+      <c r="H18" s="54"/>
+      <c r="I18" s="54"/>
+      <c r="J18" s="54"/>
+      <c r="K18" s="54"/>
+      <c r="L18" s="54"/>
+      <c r="M18" s="54"/>
+      <c r="N18" s="54"/>
+      <c r="O18" s="54"/>
+      <c r="P18" s="54"/>
+      <c r="Q18" s="54"/>
+      <c r="R18" s="54"/>
+      <c r="S18" s="1"/>
       <c r="T18" s="1"/>
       <c r="U18" s="1"/>
       <c r="V18" s="1"/>
@@ -2820,29 +2597,25 @@
       <c r="AJ18" s="1"/>
       <c r="AK18" s="1"/>
     </row>
-    <row r="19" ht="26.25" customHeight="1" spans="1:37" x14ac:dyDescent="0.25">
+    <row r="19" ht="17.25" customHeight="1" spans="1:37" x14ac:dyDescent="0.25">
       <c r="A19" s="1"/>
-      <c r="B19" s="79" t="s">
-        <v>36</v>
-      </c>
-      <c r="C19" s="67"/>
-      <c r="D19" s="80" t="s">
-        <v>37</v>
-      </c>
-      <c r="E19" s="81"/>
-      <c r="F19" s="81"/>
-      <c r="G19" s="81"/>
-      <c r="H19" s="81"/>
-      <c r="I19" s="81"/>
-      <c r="J19" s="81"/>
-      <c r="K19" s="81"/>
-      <c r="L19" s="81"/>
-      <c r="M19" s="81"/>
-      <c r="N19" s="81"/>
-      <c r="O19" s="81"/>
-      <c r="P19" s="81"/>
-      <c r="Q19" s="81"/>
-      <c r="R19" s="82"/>
+      <c r="B19" s="53"/>
+      <c r="C19" s="53"/>
+      <c r="D19" s="54"/>
+      <c r="E19" s="54"/>
+      <c r="F19" s="54"/>
+      <c r="G19" s="54"/>
+      <c r="H19" s="54"/>
+      <c r="I19" s="54"/>
+      <c r="J19" s="54"/>
+      <c r="K19" s="54"/>
+      <c r="L19" s="54"/>
+      <c r="M19" s="54"/>
+      <c r="N19" s="54"/>
+      <c r="O19" s="54"/>
+      <c r="P19" s="54"/>
+      <c r="Q19" s="54"/>
+      <c r="R19" s="54"/>
       <c r="S19" s="1"/>
       <c r="T19" s="1"/>
       <c r="U19" s="1"/>
@@ -2863,25 +2636,25 @@
       <c r="AJ19" s="1"/>
       <c r="AK19" s="1"/>
     </row>
-    <row r="20" ht="19.5" customHeight="1" spans="1:37" x14ac:dyDescent="0.25">
+    <row r="20" ht="17.25" customHeight="1" spans="1:37" x14ac:dyDescent="0.25">
       <c r="A20" s="1"/>
-      <c r="B20" s="83"/>
-      <c r="C20"/>
-      <c r="D20" s="84"/>
-      <c r="E20"/>
-      <c r="F20"/>
-      <c r="G20"/>
-      <c r="H20"/>
-      <c r="I20"/>
-      <c r="J20"/>
-      <c r="K20"/>
-      <c r="L20"/>
-      <c r="M20"/>
-      <c r="N20"/>
-      <c r="O20"/>
-      <c r="P20"/>
-      <c r="Q20"/>
-      <c r="R20" s="85"/>
+      <c r="B20" s="55"/>
+      <c r="C20" s="55"/>
+      <c r="D20" s="55"/>
+      <c r="E20" s="55"/>
+      <c r="F20" s="55"/>
+      <c r="G20" s="55"/>
+      <c r="H20" s="55"/>
+      <c r="I20" s="55"/>
+      <c r="J20" s="55"/>
+      <c r="K20" s="55"/>
+      <c r="L20" s="55"/>
+      <c r="M20" s="55"/>
+      <c r="N20" s="55"/>
+      <c r="O20" s="55"/>
+      <c r="P20" s="55"/>
+      <c r="Q20" s="55"/>
+      <c r="R20" s="55"/>
       <c r="S20" s="1"/>
       <c r="T20" s="1"/>
       <c r="U20" s="1"/>
@@ -2902,25 +2675,27 @@
       <c r="AJ20" s="1"/>
       <c r="AK20" s="1"/>
     </row>
-    <row r="21" ht="21" customHeight="1" spans="1:37" x14ac:dyDescent="0.25">
+    <row r="21" ht="17.25" customHeight="1" spans="1:37" x14ac:dyDescent="0.25">
       <c r="A21" s="1"/>
-      <c r="B21" s="83"/>
-      <c r="C21"/>
-      <c r="D21" s="84"/>
-      <c r="E21"/>
-      <c r="F21"/>
-      <c r="G21"/>
-      <c r="H21"/>
-      <c r="I21"/>
-      <c r="J21"/>
-      <c r="K21"/>
-      <c r="L21"/>
-      <c r="M21"/>
-      <c r="N21"/>
-      <c r="O21"/>
-      <c r="P21"/>
-      <c r="Q21"/>
-      <c r="R21" s="85"/>
+      <c r="B21" s="56"/>
+      <c r="C21" s="56"/>
+      <c r="D21" s="56"/>
+      <c r="E21" s="57" t="s">
+        <v>38</v>
+      </c>
+      <c r="F21" s="56"/>
+      <c r="G21" s="56"/>
+      <c r="H21" s="56"/>
+      <c r="I21" s="56"/>
+      <c r="J21" s="56"/>
+      <c r="K21" s="56"/>
+      <c r="L21" s="56"/>
+      <c r="M21" s="56"/>
+      <c r="N21" s="56"/>
+      <c r="O21" s="56"/>
+      <c r="P21" s="56"/>
+      <c r="Q21" s="56"/>
+      <c r="R21" s="56"/>
       <c r="S21" s="1"/>
       <c r="T21" s="1"/>
       <c r="U21" s="1"/>
@@ -2943,23 +2718,23 @@
     </row>
     <row r="22" ht="17.25" customHeight="1" spans="1:37" x14ac:dyDescent="0.25">
       <c r="A22" s="1"/>
-      <c r="B22" s="86"/>
-      <c r="C22" s="33"/>
-      <c r="D22" s="87"/>
-      <c r="E22" s="24"/>
-      <c r="F22" s="24"/>
-      <c r="G22" s="24"/>
-      <c r="H22" s="24"/>
-      <c r="I22" s="24"/>
-      <c r="J22" s="24"/>
-      <c r="K22" s="24"/>
-      <c r="L22" s="24"/>
-      <c r="M22" s="24"/>
-      <c r="N22" s="24"/>
-      <c r="O22" s="24"/>
-      <c r="P22" s="24"/>
-      <c r="Q22" s="24"/>
-      <c r="R22" s="88"/>
+      <c r="B22" s="56"/>
+      <c r="C22" s="56"/>
+      <c r="D22" s="56"/>
+      <c r="E22" s="56"/>
+      <c r="F22" s="56"/>
+      <c r="G22" s="56"/>
+      <c r="H22" s="56"/>
+      <c r="I22" s="56"/>
+      <c r="J22" s="56"/>
+      <c r="K22" s="56"/>
+      <c r="L22" s="56"/>
+      <c r="M22" s="56"/>
+      <c r="N22" s="56"/>
+      <c r="O22" s="56"/>
+      <c r="P22" s="56"/>
+      <c r="Q22" s="56"/>
+      <c r="R22" s="56"/>
       <c r="S22" s="1"/>
       <c r="T22" s="1"/>
       <c r="U22" s="1"/>
@@ -2982,23 +2757,23 @@
     </row>
     <row r="23" ht="17.25" customHeight="1" spans="1:37" x14ac:dyDescent="0.25">
       <c r="A23" s="1"/>
-      <c r="B23" s="89"/>
-      <c r="C23" s="89"/>
-      <c r="D23" s="89"/>
-      <c r="E23" s="89"/>
-      <c r="F23" s="89"/>
-      <c r="G23" s="89"/>
-      <c r="H23" s="89"/>
-      <c r="I23" s="89"/>
-      <c r="J23" s="89"/>
-      <c r="K23" s="89"/>
-      <c r="L23" s="89"/>
-      <c r="M23" s="89"/>
-      <c r="N23" s="89"/>
-      <c r="O23" s="89"/>
-      <c r="P23" s="89"/>
-      <c r="Q23" s="89"/>
-      <c r="R23" s="89"/>
+      <c r="B23" s="56"/>
+      <c r="C23" s="56"/>
+      <c r="D23" s="56"/>
+      <c r="E23" s="56"/>
+      <c r="F23" s="56"/>
+      <c r="G23" s="56"/>
+      <c r="H23" s="56"/>
+      <c r="I23" s="56"/>
+      <c r="J23" s="56"/>
+      <c r="K23" s="56"/>
+      <c r="L23" s="56"/>
+      <c r="M23" s="56"/>
+      <c r="N23" s="56"/>
+      <c r="O23" s="56"/>
+      <c r="P23" s="56"/>
+      <c r="Q23" s="56"/>
+      <c r="R23" s="56"/>
       <c r="S23" s="1"/>
       <c r="T23" s="1"/>
       <c r="U23" s="1"/>
@@ -3021,25 +2796,23 @@
     </row>
     <row r="24" ht="17.25" customHeight="1" spans="1:37" x14ac:dyDescent="0.25">
       <c r="A24" s="1"/>
-      <c r="B24" s="90"/>
-      <c r="C24" s="90"/>
-      <c r="D24" s="90"/>
-      <c r="E24" s="91" t="s">
-        <v>38</v>
-      </c>
-      <c r="F24" s="90"/>
-      <c r="G24" s="90"/>
-      <c r="H24" s="90"/>
-      <c r="I24" s="90"/>
-      <c r="J24" s="90"/>
-      <c r="K24" s="90"/>
-      <c r="L24" s="90"/>
-      <c r="M24" s="90"/>
-      <c r="N24" s="90"/>
-      <c r="O24" s="90"/>
-      <c r="P24" s="90"/>
-      <c r="Q24" s="90"/>
-      <c r="R24" s="90"/>
+      <c r="B24" s="56"/>
+      <c r="C24" s="56"/>
+      <c r="D24" s="56"/>
+      <c r="E24" s="56"/>
+      <c r="F24" s="56"/>
+      <c r="G24" s="56"/>
+      <c r="H24" s="56"/>
+      <c r="I24" s="56"/>
+      <c r="J24" s="56"/>
+      <c r="K24" s="56"/>
+      <c r="L24" s="56"/>
+      <c r="M24" s="56"/>
+      <c r="N24" s="56"/>
+      <c r="O24" s="56"/>
+      <c r="P24" s="56"/>
+      <c r="Q24" s="56"/>
+      <c r="R24" s="56"/>
       <c r="S24" s="1"/>
       <c r="T24" s="1"/>
       <c r="U24" s="1"/>
@@ -3060,125 +2833,8 @@
       <c r="AJ24" s="1"/>
       <c r="AK24" s="1"/>
     </row>
-    <row r="25" ht="17.25" customHeight="1" spans="1:37" x14ac:dyDescent="0.25">
-      <c r="A25" s="1"/>
-      <c r="B25" s="90"/>
-      <c r="C25" s="90"/>
-      <c r="D25" s="90"/>
-      <c r="E25" s="90"/>
-      <c r="F25" s="90"/>
-      <c r="G25" s="90"/>
-      <c r="H25" s="90"/>
-      <c r="I25" s="90"/>
-      <c r="J25" s="90"/>
-      <c r="K25" s="90"/>
-      <c r="L25" s="90"/>
-      <c r="M25" s="90"/>
-      <c r="N25" s="90"/>
-      <c r="O25" s="90"/>
-      <c r="P25" s="90"/>
-      <c r="Q25" s="90"/>
-      <c r="R25" s="90"/>
-      <c r="S25" s="1"/>
-      <c r="T25" s="1"/>
-      <c r="U25" s="1"/>
-      <c r="V25" s="1"/>
-      <c r="W25" s="1"/>
-      <c r="X25" s="1"/>
-      <c r="Y25" s="1"/>
-      <c r="Z25" s="1"/>
-      <c r="AA25" s="1"/>
-      <c r="AB25" s="1"/>
-      <c r="AC25" s="1"/>
-      <c r="AD25" s="1"/>
-      <c r="AE25" s="1"/>
-      <c r="AF25" s="1"/>
-      <c r="AG25" s="1"/>
-      <c r="AH25" s="1"/>
-      <c r="AI25" s="1"/>
-      <c r="AJ25" s="1"/>
-      <c r="AK25" s="1"/>
-    </row>
-    <row r="26" ht="17.25" customHeight="1" spans="1:37" x14ac:dyDescent="0.25">
-      <c r="A26" s="1"/>
-      <c r="B26" s="90"/>
-      <c r="C26" s="90"/>
-      <c r="D26" s="90"/>
-      <c r="E26" s="90"/>
-      <c r="F26" s="90"/>
-      <c r="G26" s="90"/>
-      <c r="H26" s="90"/>
-      <c r="I26" s="90"/>
-      <c r="J26" s="90"/>
-      <c r="K26" s="90"/>
-      <c r="L26" s="90"/>
-      <c r="M26" s="90"/>
-      <c r="N26" s="90"/>
-      <c r="O26" s="90"/>
-      <c r="P26" s="90"/>
-      <c r="Q26" s="90"/>
-      <c r="R26" s="90"/>
-      <c r="S26" s="1"/>
-      <c r="T26" s="1"/>
-      <c r="U26" s="1"/>
-      <c r="V26" s="1"/>
-      <c r="W26" s="1"/>
-      <c r="X26" s="1"/>
-      <c r="Y26" s="1"/>
-      <c r="Z26" s="1"/>
-      <c r="AA26" s="1"/>
-      <c r="AB26" s="1"/>
-      <c r="AC26" s="1"/>
-      <c r="AD26" s="1"/>
-      <c r="AE26" s="1"/>
-      <c r="AF26" s="1"/>
-      <c r="AG26" s="1"/>
-      <c r="AH26" s="1"/>
-      <c r="AI26" s="1"/>
-      <c r="AJ26" s="1"/>
-      <c r="AK26" s="1"/>
-    </row>
-    <row r="27" ht="17.25" customHeight="1" spans="1:37" x14ac:dyDescent="0.25">
-      <c r="A27" s="1"/>
-      <c r="B27" s="90"/>
-      <c r="C27" s="90"/>
-      <c r="D27" s="90"/>
-      <c r="E27" s="90"/>
-      <c r="F27" s="90"/>
-      <c r="G27" s="90"/>
-      <c r="H27" s="90"/>
-      <c r="I27" s="90"/>
-      <c r="J27" s="90"/>
-      <c r="K27" s="90"/>
-      <c r="L27" s="90"/>
-      <c r="M27" s="90"/>
-      <c r="N27" s="90"/>
-      <c r="O27" s="90"/>
-      <c r="P27" s="90"/>
-      <c r="Q27" s="90"/>
-      <c r="R27" s="90"/>
-      <c r="S27" s="1"/>
-      <c r="T27" s="1"/>
-      <c r="U27" s="1"/>
-      <c r="V27" s="1"/>
-      <c r="W27" s="1"/>
-      <c r="X27" s="1"/>
-      <c r="Y27" s="1"/>
-      <c r="Z27" s="1"/>
-      <c r="AA27" s="1"/>
-      <c r="AB27" s="1"/>
-      <c r="AC27" s="1"/>
-      <c r="AD27" s="1"/>
-      <c r="AE27" s="1"/>
-      <c r="AF27" s="1"/>
-      <c r="AG27" s="1"/>
-      <c r="AH27" s="1"/>
-      <c r="AI27" s="1"/>
-      <c r="AJ27" s="1"/>
-      <c r="AK27" s="1"/>
-    </row>
   </sheetData>
-  <mergeCells count="48">
+  <mergeCells count="33">
     <mergeCell ref="B1:R2"/>
     <mergeCell ref="D6:F6"/>
     <mergeCell ref="J6:K6"/>
@@ -3210,27 +2866,12 @@
     <mergeCell ref="I15:J15"/>
     <mergeCell ref="K15:N15"/>
     <mergeCell ref="O15:R15"/>
-    <mergeCell ref="B16:E16"/>
-    <mergeCell ref="F16:G16"/>
-    <mergeCell ref="I16:J16"/>
-    <mergeCell ref="K16:N16"/>
-    <mergeCell ref="O16:R16"/>
-    <mergeCell ref="B17:E17"/>
-    <mergeCell ref="F17:G17"/>
-    <mergeCell ref="I17:J17"/>
-    <mergeCell ref="K17:N17"/>
-    <mergeCell ref="O17:R17"/>
-    <mergeCell ref="B18:E18"/>
-    <mergeCell ref="F18:G18"/>
-    <mergeCell ref="I18:J18"/>
-    <mergeCell ref="K18:N18"/>
-    <mergeCell ref="O18:R18"/>
-    <mergeCell ref="B19:C22"/>
-    <mergeCell ref="D19:R22"/>
+    <mergeCell ref="B16:C19"/>
+    <mergeCell ref="D16:R19"/>
   </mergeCells>
   <printOptions horizontalCentered="1"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0" footer="0"/>
-  <pageSetup paperSize="9" orientation="landscape" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="0" firstPageNumber="1" useFirstPageNumber="1" copies="1"/>
+  <pageSetup paperSize="9" orientation="landscape" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1" firstPageNumber="1" useFirstPageNumber="1" copies="1"/>
   <drawing r:id="rId1"/>
 </worksheet>
 </file>
@@ -3276,23 +2917,23 @@
     </row>
     <row r="3" ht="30" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A3" s="1"/>
-      <c r="B3" s="92" t="s">
+      <c r="B3" s="58" t="s">
         <v>39</v>
       </c>
-      <c r="C3" s="93" t="s">
+      <c r="C3" s="59" t="s">
         <v>40</v>
       </c>
-      <c r="D3" s="94"/>
-      <c r="E3" s="94"/>
-      <c r="F3" s="94"/>
-      <c r="G3" s="94"/>
-      <c r="H3" s="94"/>
-      <c r="I3" s="94"/>
-      <c r="J3" s="94"/>
-      <c r="K3" s="94"/>
-      <c r="L3" s="94"/>
-      <c r="M3" s="94"/>
-      <c r="N3" s="95"/>
+      <c r="D3" s="60"/>
+      <c r="E3" s="60"/>
+      <c r="F3" s="60"/>
+      <c r="G3" s="60"/>
+      <c r="H3" s="60"/>
+      <c r="I3" s="60"/>
+      <c r="J3" s="60"/>
+      <c r="K3" s="60"/>
+      <c r="L3" s="60"/>
+      <c r="M3" s="60"/>
+      <c r="N3" s="61"/>
     </row>
     <row r="4" ht="15" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A4" s="1"/>
@@ -3302,69 +2943,69 @@
     </row>
     <row r="5" ht="31.5" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A5" s="1"/>
-      <c r="B5" s="96" t="s">
+      <c r="B5" s="62" t="s">
         <v>27</v>
       </c>
-      <c r="C5" s="97" t="s">
+      <c r="C5" s="63" t="s">
         <v>28</v>
       </c>
-      <c r="D5" s="97" t="s">
+      <c r="D5" s="63" t="s">
         <v>41</v>
       </c>
-      <c r="E5" s="97" t="s">
+      <c r="E5" s="63" t="s">
         <v>29</v>
       </c>
-      <c r="F5" s="52" t="s">
+      <c r="F5" s="42" t="s">
         <v>42</v>
       </c>
-      <c r="G5" s="51"/>
-      <c r="H5" s="98" t="s">
+      <c r="G5" s="64"/>
+      <c r="H5" s="65" t="s">
         <v>43</v>
       </c>
-      <c r="I5" s="99"/>
-      <c r="J5" s="52" t="s">
+      <c r="I5" s="66"/>
+      <c r="J5" s="42" t="s">
         <v>44</v>
       </c>
-      <c r="K5" s="51"/>
-      <c r="L5" s="98" t="s">
+      <c r="K5" s="64"/>
+      <c r="L5" s="65" t="s">
         <v>45</v>
       </c>
-      <c r="M5" s="99"/>
-      <c r="N5" s="52" t="s">
+      <c r="M5" s="66"/>
+      <c r="N5" s="42" t="s">
         <v>32</v>
       </c>
     </row>
     <row r="6" ht="30.75" customHeight="1" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A6" s="1"/>
-      <c r="B6" s="100"/>
-      <c r="C6" s="101"/>
-      <c r="D6" s="101"/>
-      <c r="E6" s="101"/>
-      <c r="F6" s="102" t="s">
+      <c r="B6" s="67"/>
+      <c r="C6" s="68"/>
+      <c r="D6" s="68"/>
+      <c r="E6" s="68"/>
+      <c r="F6" s="69" t="s">
         <v>30</v>
       </c>
-      <c r="G6" s="103" t="s">
+      <c r="G6" s="70" t="s">
         <v>31</v>
       </c>
-      <c r="H6" s="101" t="s">
+      <c r="H6" s="68" t="s">
         <v>30</v>
       </c>
-      <c r="I6" s="104" t="s">
+      <c r="I6" s="71" t="s">
         <v>31</v>
       </c>
-      <c r="J6" s="102" t="s">
+      <c r="J6" s="69" t="s">
         <v>30</v>
       </c>
-      <c r="K6" s="103" t="s">
+      <c r="K6" s="70" t="s">
         <v>31</v>
       </c>
-      <c r="L6" s="105" t="s">
+      <c r="L6" s="72" t="s">
         <v>30</v>
       </c>
-      <c r="M6" s="104" t="s">
+      <c r="M6" s="71" t="s">
         <v>31</v>
       </c>
-      <c r="N6" s="106"/>
+      <c r="N6" s="73"/>
       <c r="O6" s="1"/>
       <c r="P6" s="1"/>
       <c r="Q6" s="1"/>
@@ -3372,430 +3013,430 @@
     </row>
     <row r="7" ht="30" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A7" s="1"/>
-      <c r="B7" s="107" t="s">
+      <c r="B7" s="74" t="s">
         <v>46</v>
       </c>
-      <c r="C7" s="108" t="s">
+      <c r="C7" s="75" t="s">
         <v>47</v>
       </c>
-      <c r="D7" s="109" t="s">
+      <c r="D7" s="76" t="s">
         <v>48</v>
       </c>
-      <c r="E7" s="110">
+      <c r="E7" s="77">
         <v>100</v>
       </c>
-      <c r="F7" s="111">
+      <c r="F7" s="78">
         <v>12000</v>
       </c>
-      <c r="G7" s="110">
+      <c r="G7" s="77">
         <f>E7*F7</f>
       </c>
-      <c r="H7" s="111">
+      <c r="H7" s="78">
         <v>8000</v>
       </c>
-      <c r="I7" s="110">
+      <c r="I7" s="77">
         <f>E7*H7</f>
       </c>
-      <c r="J7" s="111">
+      <c r="J7" s="78">
         <v>2000</v>
       </c>
-      <c r="K7" s="111">
+      <c r="K7" s="78">
         <f>E7*J7</f>
       </c>
-      <c r="L7" s="112">
+      <c r="L7" s="79">
         <f>F7+H7+J7</f>
       </c>
-      <c r="M7" s="110">
+      <c r="M7" s="77">
         <f>G7+I7+K7</f>
       </c>
-      <c r="N7" s="109"/>
-    </row>
-    <row r="8" ht="20" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="N7" s="76"/>
+    </row>
+    <row r="8" ht="24" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A8" s="1"/>
-      <c r="B8" s="113" t="s">
+      <c r="B8" s="80" t="s">
         <v>49</v>
       </c>
-      <c r="C8" s="108" t="s">
+      <c r="C8" s="75" t="s">
         <v>47</v>
       </c>
-      <c r="D8" s="114" t="s">
+      <c r="D8" s="81" t="s">
         <v>48</v>
       </c>
-      <c r="E8" s="110">
+      <c r="E8" s="77">
         <v>105</v>
       </c>
-      <c r="F8" s="111">
+      <c r="F8" s="78">
         <v>12500</v>
       </c>
-      <c r="G8" s="110">
+      <c r="G8" s="77">
         <f>E8*F8</f>
       </c>
-      <c r="H8" s="111">
+      <c r="H8" s="78">
         <v>8000</v>
       </c>
-      <c r="I8" s="110">
+      <c r="I8" s="77">
         <f>E8*H8</f>
       </c>
-      <c r="J8" s="111">
+      <c r="J8" s="78">
         <v>2000</v>
       </c>
-      <c r="K8" s="111">
+      <c r="K8" s="78">
         <f>E8*J8</f>
       </c>
-      <c r="L8" s="112">
+      <c r="L8" s="79">
         <f>F8+H8+J8</f>
       </c>
-      <c r="M8" s="110">
+      <c r="M8" s="77">
         <f>G8+I8+K8</f>
       </c>
-      <c r="N8" s="109"/>
+      <c r="N8" s="76"/>
     </row>
     <row r="9" ht="30" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A9" s="1"/>
-      <c r="B9" s="115" t="s">
+      <c r="B9" s="82" t="s">
         <v>50</v>
       </c>
-      <c r="C9" s="116" t="s">
+      <c r="C9" s="83" t="s">
         <v>47</v>
       </c>
-      <c r="D9" s="109" t="s">
+      <c r="D9" s="76" t="s">
         <v>48</v>
       </c>
-      <c r="E9" s="110">
+      <c r="E9" s="77">
         <v>110</v>
       </c>
-      <c r="F9" s="111">
+      <c r="F9" s="78">
         <v>13000</v>
       </c>
-      <c r="G9" s="110">
+      <c r="G9" s="77">
         <f>E9*F9</f>
       </c>
-      <c r="H9" s="111">
+      <c r="H9" s="78">
         <v>8000</v>
       </c>
-      <c r="I9" s="110">
+      <c r="I9" s="77">
         <f>E9*H9</f>
       </c>
-      <c r="J9" s="111">
+      <c r="J9" s="78">
         <v>2000</v>
       </c>
-      <c r="K9" s="111">
+      <c r="K9" s="78">
         <f>E9*J9</f>
       </c>
-      <c r="L9" s="112">
+      <c r="L9" s="79">
         <f>F9+H9+J9</f>
       </c>
-      <c r="M9" s="110">
+      <c r="M9" s="77">
         <f>G9+I9+K9</f>
       </c>
-      <c r="N9" s="109"/>
+      <c r="N9" s="76"/>
     </row>
     <row r="10" ht="30" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A10" s="1"/>
-      <c r="B10" s="115" t="s">
+      <c r="B10" s="82" t="s">
         <v>51</v>
       </c>
-      <c r="C10" s="116" t="s">
+      <c r="C10" s="83" t="s">
         <v>47</v>
       </c>
-      <c r="D10" s="109" t="s">
+      <c r="D10" s="76" t="s">
         <v>48</v>
       </c>
-      <c r="E10" s="110">
+      <c r="E10" s="77">
         <v>115</v>
       </c>
-      <c r="F10" s="111">
+      <c r="F10" s="78">
         <v>13500</v>
       </c>
-      <c r="G10" s="110">
+      <c r="G10" s="77">
         <f>E10*F10</f>
       </c>
-      <c r="H10" s="111">
+      <c r="H10" s="78">
         <v>8000</v>
       </c>
-      <c r="I10" s="110">
+      <c r="I10" s="77">
         <f>E10*H10</f>
       </c>
-      <c r="J10" s="111">
+      <c r="J10" s="78">
         <v>2000</v>
       </c>
-      <c r="K10" s="110">
+      <c r="K10" s="77">
         <f>E10*J10</f>
       </c>
-      <c r="L10" s="112">
+      <c r="L10" s="79">
         <f>F10+H10+J10</f>
       </c>
-      <c r="M10" s="110">
+      <c r="M10" s="77">
         <f>G10+I10+K10</f>
       </c>
-      <c r="N10" s="109"/>
-    </row>
-    <row r="11" ht="20" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="N10" s="76"/>
+    </row>
+    <row r="11" ht="24" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A11" s="1"/>
-      <c r="B11" s="115" t="s">
+      <c r="B11" s="82" t="s">
         <v>52</v>
       </c>
-      <c r="C11" s="116" t="s">
+      <c r="C11" s="83" t="s">
         <v>47</v>
       </c>
-      <c r="D11" s="109" t="s">
+      <c r="D11" s="76" t="s">
         <v>48</v>
       </c>
-      <c r="E11" s="110">
+      <c r="E11" s="77">
         <v>120</v>
       </c>
-      <c r="F11" s="111">
+      <c r="F11" s="78">
         <v>14000</v>
       </c>
-      <c r="G11" s="110">
+      <c r="G11" s="77">
         <f>E11*F11</f>
       </c>
-      <c r="H11" s="111">
+      <c r="H11" s="78">
         <v>8000</v>
       </c>
-      <c r="I11" s="110">
+      <c r="I11" s="77">
         <f>E11*H11</f>
       </c>
-      <c r="J11" s="111">
+      <c r="J11" s="78">
         <v>2000</v>
       </c>
-      <c r="K11" s="111">
+      <c r="K11" s="78">
         <f>E11*J11</f>
       </c>
-      <c r="L11" s="112">
+      <c r="L11" s="79">
         <f>F11+H11+J11</f>
       </c>
-      <c r="M11" s="110">
+      <c r="M11" s="77">
         <f>G11+I11+K11</f>
       </c>
-      <c r="N11" s="109"/>
+      <c r="N11" s="76"/>
     </row>
     <row r="12" ht="30" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A12" s="1"/>
-      <c r="B12" s="115" t="s">
+      <c r="B12" s="82" t="s">
         <v>53</v>
       </c>
-      <c r="C12" s="116" t="s">
+      <c r="C12" s="83" t="s">
         <v>47</v>
       </c>
-      <c r="D12" s="109" t="s">
+      <c r="D12" s="76" t="s">
         <v>48</v>
       </c>
-      <c r="E12" s="110">
+      <c r="E12" s="77">
         <v>125</v>
       </c>
-      <c r="F12" s="111">
+      <c r="F12" s="78">
         <v>14500</v>
       </c>
-      <c r="G12" s="110">
+      <c r="G12" s="77">
         <f>E12*F12</f>
       </c>
-      <c r="H12" s="111">
+      <c r="H12" s="78">
         <v>8000</v>
       </c>
-      <c r="I12" s="110">
+      <c r="I12" s="77">
         <f>E12*H12</f>
       </c>
-      <c r="J12" s="111">
+      <c r="J12" s="78">
         <v>2000</v>
       </c>
-      <c r="K12" s="110">
+      <c r="K12" s="77">
         <f>E12*J12</f>
       </c>
-      <c r="L12" s="112">
+      <c r="L12" s="79">
         <f>F12+H12+J12</f>
       </c>
-      <c r="M12" s="110">
+      <c r="M12" s="77">
         <f>G12+I12+K12</f>
       </c>
-      <c r="N12" s="109"/>
+      <c r="N12" s="76"/>
     </row>
     <row r="13" ht="30" customHeight="1" spans="2:14" x14ac:dyDescent="0.25">
-      <c r="B13" s="115" t="s">
+      <c r="B13" s="82" t="s">
         <v>54</v>
       </c>
-      <c r="C13" s="116" t="s">
+      <c r="C13" s="83" t="s">
         <v>47</v>
       </c>
-      <c r="D13" s="109" t="s">
+      <c r="D13" s="76" t="s">
         <v>48</v>
       </c>
-      <c r="E13" s="110">
+      <c r="E13" s="77">
         <v>130</v>
       </c>
-      <c r="F13" s="111">
+      <c r="F13" s="78">
         <v>15000</v>
       </c>
-      <c r="G13" s="110">
+      <c r="G13" s="77">
         <f>E13*F13</f>
       </c>
-      <c r="H13" s="111">
+      <c r="H13" s="78">
         <v>8000</v>
       </c>
-      <c r="I13" s="110">
+      <c r="I13" s="77">
         <f>E13*H13</f>
       </c>
-      <c r="J13" s="111">
+      <c r="J13" s="78">
         <v>2000</v>
       </c>
-      <c r="K13" s="110">
+      <c r="K13" s="77">
         <f>E13*J13</f>
       </c>
-      <c r="L13" s="112">
+      <c r="L13" s="79">
         <f>F13+H13+J13</f>
       </c>
-      <c r="M13" s="110">
+      <c r="M13" s="77">
         <f>G13+I13+K13</f>
       </c>
-      <c r="N13" s="109"/>
+      <c r="N13" s="76"/>
     </row>
     <row r="14" ht="30" customHeight="1" spans="2:14" x14ac:dyDescent="0.25">
-      <c r="B14" s="115" t="s">
+      <c r="B14" s="82" t="s">
         <v>55</v>
       </c>
-      <c r="C14" s="116" t="s">
+      <c r="C14" s="83" t="s">
         <v>47</v>
       </c>
-      <c r="D14" s="109" t="s">
+      <c r="D14" s="76" t="s">
         <v>48</v>
       </c>
-      <c r="E14" s="110">
+      <c r="E14" s="77">
         <v>135</v>
       </c>
-      <c r="F14" s="111">
+      <c r="F14" s="78">
         <v>15500</v>
       </c>
-      <c r="G14" s="110">
+      <c r="G14" s="77">
         <f>E14*F14</f>
       </c>
-      <c r="H14" s="111">
+      <c r="H14" s="78">
         <v>8000</v>
       </c>
-      <c r="I14" s="110">
+      <c r="I14" s="77">
         <f>E14*H14</f>
       </c>
-      <c r="J14" s="111">
+      <c r="J14" s="78">
         <v>2000</v>
       </c>
-      <c r="K14" s="111">
+      <c r="K14" s="78">
         <f>E14*J14</f>
       </c>
-      <c r="L14" s="112">
+      <c r="L14" s="79">
         <f>F14+H14+J14</f>
       </c>
-      <c r="M14" s="110">
+      <c r="M14" s="77">
         <f>G14+I14+K14</f>
       </c>
-      <c r="N14" s="109"/>
+      <c r="N14" s="76"/>
     </row>
     <row r="15" ht="30" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="B15" s="117" t="s">
+      <c r="B15" s="84" t="s">
         <v>56</v>
       </c>
-      <c r="C15" s="118"/>
-      <c r="D15" s="119"/>
-      <c r="E15" s="120"/>
-      <c r="F15" s="120"/>
-      <c r="G15" s="121">
+      <c r="C15" s="85"/>
+      <c r="D15" s="86"/>
+      <c r="E15" s="87"/>
+      <c r="F15" s="87"/>
+      <c r="G15" s="88">
         <f>SUM(G7:G14)</f>
       </c>
-      <c r="H15" s="122"/>
-      <c r="I15" s="121">
+      <c r="H15" s="89"/>
+      <c r="I15" s="88">
         <f>SUM(I7:I14)</f>
       </c>
-      <c r="J15" s="120"/>
-      <c r="K15" s="121">
+      <c r="J15" s="87"/>
+      <c r="K15" s="88">
         <f>SUM(K7:K14)</f>
       </c>
-      <c r="L15" s="120"/>
-      <c r="M15" s="120">
+      <c r="L15" s="87"/>
+      <c r="M15" s="87">
         <f>SUM(M7:M14)</f>
       </c>
-      <c r="N15" s="123"/>
+      <c r="N15" s="90"/>
     </row>
     <row r="16" ht="17.25" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="B16" s="124" t="s">
+      <c r="B16" s="91" t="s">
         <v>57</v>
       </c>
-      <c r="C16" s="116"/>
-      <c r="D16" s="109" t="s">
+      <c r="C16" s="83"/>
+      <c r="D16" s="76" t="s">
         <v>58</v>
       </c>
-      <c r="E16" s="110">
+      <c r="E16" s="77">
         <v>3</v>
       </c>
-      <c r="F16" s="110"/>
-      <c r="G16" s="110"/>
-      <c r="H16" s="110"/>
-      <c r="I16" s="110"/>
-      <c r="J16" s="110"/>
-      <c r="K16" s="110"/>
-      <c r="L16" s="112"/>
-      <c r="M16" s="110">
+      <c r="F16" s="77"/>
+      <c r="G16" s="77"/>
+      <c r="H16" s="77"/>
+      <c r="I16" s="77"/>
+      <c r="J16" s="77"/>
+      <c r="K16" s="77"/>
+      <c r="L16" s="79"/>
+      <c r="M16" s="77">
         <f>M15*0.03</f>
       </c>
-      <c r="N16" s="109"/>
+      <c r="N16" s="76"/>
     </row>
     <row r="17" ht="30" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="B17" s="55" t="s">
+      <c r="B17" s="44" t="s">
         <v>59</v>
       </c>
-      <c r="C17" s="116"/>
-      <c r="D17" s="109" t="s">
+      <c r="C17" s="83"/>
+      <c r="D17" s="76" t="s">
         <v>58</v>
       </c>
-      <c r="E17" s="110">
+      <c r="E17" s="77">
         <v>6</v>
       </c>
-      <c r="F17" s="110"/>
-      <c r="G17" s="110"/>
-      <c r="H17" s="110"/>
-      <c r="I17" s="110"/>
-      <c r="J17" s="110"/>
-      <c r="K17" s="110"/>
-      <c r="L17" s="112"/>
-      <c r="M17" s="110">
+      <c r="F17" s="77"/>
+      <c r="G17" s="77"/>
+      <c r="H17" s="77"/>
+      <c r="I17" s="77"/>
+      <c r="J17" s="77"/>
+      <c r="K17" s="77"/>
+      <c r="L17" s="79"/>
+      <c r="M17" s="77">
         <f>M15*0.06</f>
       </c>
-      <c r="N17" s="109"/>
+      <c r="N17" s="76"/>
     </row>
     <row r="18" ht="30" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="B18" s="125" t="s">
+      <c r="B18" s="92" t="s">
         <v>60</v>
       </c>
-      <c r="C18" s="126"/>
-      <c r="D18" s="123"/>
-      <c r="E18" s="123"/>
-      <c r="F18" s="127"/>
-      <c r="G18" s="121"/>
-      <c r="H18" s="123"/>
-      <c r="I18" s="121"/>
-      <c r="J18" s="123"/>
-      <c r="K18" s="121"/>
-      <c r="L18" s="123"/>
-      <c r="M18" s="121">
+      <c r="C18" s="93"/>
+      <c r="D18" s="90"/>
+      <c r="E18" s="90"/>
+      <c r="F18" s="94"/>
+      <c r="G18" s="88"/>
+      <c r="H18" s="90"/>
+      <c r="I18" s="88"/>
+      <c r="J18" s="90"/>
+      <c r="K18" s="88"/>
+      <c r="L18" s="90"/>
+      <c r="M18" s="88">
         <f>SUM(M15:M17)</f>
       </c>
-      <c r="N18" s="123"/>
+      <c r="N18" s="90"/>
     </row>
     <row r="19" ht="30" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="B19" s="128" t="s">
+      <c r="B19" s="95" t="s">
         <v>61</v>
       </c>
-      <c r="C19" s="129"/>
-      <c r="D19" s="123"/>
-      <c r="E19" s="123"/>
-      <c r="F19" s="127"/>
-      <c r="G19" s="123"/>
-      <c r="H19" s="123"/>
-      <c r="I19" s="123"/>
-      <c r="J19" s="123"/>
-      <c r="K19" s="123"/>
-      <c r="L19" s="123"/>
-      <c r="M19" s="130">
+      <c r="C19" s="96"/>
+      <c r="D19" s="90"/>
+      <c r="E19" s="90"/>
+      <c r="F19" s="94"/>
+      <c r="G19" s="90"/>
+      <c r="H19" s="90"/>
+      <c r="I19" s="90"/>
+      <c r="J19" s="90"/>
+      <c r="K19" s="90"/>
+      <c r="L19" s="90"/>
+      <c r="M19" s="97">
         <f>FLOOR(M18,100000)</f>
       </c>
-      <c r="N19" s="131" t="s">
+      <c r="N19" s="98" t="s">
         <v>62</v>
       </c>
     </row>

</xml_diff>

<commit_message>
fix(excel/c14): 을지 fitToHeight=2 — 3페이지 분할 방지 + 샘플 재생성
c12/c13 행 높이 증가 효과로 sample-2 (11행) 의 을지가 PDF 변환 시
3페이지로 분할되는 UAT 이슈 발생.

수정: enforceLandscape 의 detail 분기를 fitToHeight=0(무제한) → 2(최대 2페이지).
fitToWidth=1 유지 → 가로 1페이지 + 세로 2페이지 자동 축소.

검증: sample-2 을지 pageSetup → fitToHeight=2, scale=71 자동 산정됨
      (Excel/LibreOffice 가 2페이지 캡 적용 시 동적 축소).

c13 의 행 높이 한글 폭 교정 효과도 함께 샘플에 반영:
  - "줄눈·크랙 실란트 보강포" C:/Program Files/Git/ "이중복합시트 3.8mm" 모두 h=42 (2줄)
</commit_message>
<xml_diff>
--- a/samples/sample-1-basic-8rows.xlsx
+++ b/samples/sample-1-basic-8rows.xlsx
@@ -3051,7 +3051,7 @@
       </c>
       <c r="N7" s="76"/>
     </row>
-    <row r="8" ht="24" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="8" ht="42" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A8" s="1"/>
       <c r="B8" s="80" t="s">
         <v>49</v>
@@ -3091,7 +3091,7 @@
       </c>
       <c r="N8" s="76"/>
     </row>
-    <row r="9" ht="30" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="9" ht="42" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A9" s="1"/>
       <c r="B9" s="82" t="s">
         <v>50</v>
@@ -3171,7 +3171,7 @@
       </c>
       <c r="N10" s="76"/>
     </row>
-    <row r="11" ht="24" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="11" ht="42" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A11" s="1"/>
       <c r="B11" s="82" t="s">
         <v>52</v>
@@ -3452,7 +3452,7 @@
   </mergeCells>
   <printOptions horizontalCentered="1"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0" footer="0"/>
-  <pageSetup paperSize="9" orientation="landscape" horizontalDpi="4294967295" verticalDpi="4294967295" scale="71" fitToWidth="1" fitToHeight="0" firstPageNumber="1" useFirstPageNumber="1" copies="1"/>
+  <pageSetup paperSize="9" orientation="landscape" horizontalDpi="4294967295" verticalDpi="4294967295" scale="71" fitToWidth="1" fitToHeight="2" firstPageNumber="1" useFirstPageNumber="1" copies="1"/>
   <drawing r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
fix(excel/c15): 을지 행 높이 계수 축소 + scale -10 마진
c14 의 fitToHeight=2 만으로는 행 높이 증가 효과 미반영으로
sample-2 를 2페이지에 못 담는 UAT 잔존 이슈.

A. 행 높이 공식 계수 축소:
   lines * 18 + 6  →  lines * 15 + 4
   2줄 한글 품명: 42 → 34 (≈19% 감소)
   sample-2 11행 합계 약 30pt (1행분) 절감.

B. 을지 scale 추가 마진:
   exceljs 는 scale 자동 산정을 하지 않음 (writeBuffer 로 mutate 안 됨).
   ws.pageSetup.scale 은 템플릿 저장값 (complex.xlsx Sheet2 = 71).
   enforceLandscape detail 분기에서:
     scale = max(60, base.scale - 10)   // 71 → 61
   LibreOffice / Google Sheets 의 fitToHeight 해석 차이 보정.

검증 (sample-2):
  - r8/r9/r11 (2줄): h=42 → 34 ✓
  - Sheet2 pageSetup: scale=61, fitToHeight=2 ✓
  - 회귀 테스트 통과 ✓

머지 블로커: PM 환경 (MS Excel "인쇄 미리보기" 또는 LibreOffice
soffice --convert-to pdf) 에서 sample-2 페이지 수 = 2 + 2줄 표시 유지.
</commit_message>
<xml_diff>
--- a/samples/sample-1-basic-8rows.xlsx
+++ b/samples/sample-1-basic-8rows.xlsx
@@ -3051,7 +3051,7 @@
       </c>
       <c r="N7" s="76"/>
     </row>
-    <row r="8" ht="42" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="8" ht="34" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A8" s="1"/>
       <c r="B8" s="80" t="s">
         <v>49</v>
@@ -3091,7 +3091,7 @@
       </c>
       <c r="N8" s="76"/>
     </row>
-    <row r="9" ht="42" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="9" ht="34" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A9" s="1"/>
       <c r="B9" s="82" t="s">
         <v>50</v>
@@ -3171,7 +3171,7 @@
       </c>
       <c r="N10" s="76"/>
     </row>
-    <row r="11" ht="42" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="11" ht="34" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A11" s="1"/>
       <c r="B11" s="82" t="s">
         <v>52</v>
@@ -3452,7 +3452,7 @@
   </mergeCells>
   <printOptions horizontalCentered="1"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0" footer="0"/>
-  <pageSetup paperSize="9" orientation="landscape" horizontalDpi="4294967295" verticalDpi="4294967295" scale="71" fitToWidth="1" fitToHeight="2" firstPageNumber="1" useFirstPageNumber="1" copies="1"/>
+  <pageSetup paperSize="9" orientation="landscape" horizontalDpi="4294967295" verticalDpi="4294967295" scale="61" fitToWidth="1" fitToHeight="2" firstPageNumber="1" useFirstPageNumber="1" copies="1"/>
   <drawing r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>